<commit_message>
Update the new main results tables
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Additional comparative analyses.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Additional comparative analyses.xlsx
@@ -73,148 +73,148 @@
     <t>0 (0.0-0.0)</t>
   </si>
   <si>
-    <t>764 (236-1,449)</t>
-  </si>
-  <si>
-    <t>1,144 (409-2,493)</t>
-  </si>
-  <si>
-    <t>1,464 (542-3,254)</t>
-  </si>
-  <si>
-    <t>777 (246-1,633)</t>
-  </si>
-  <si>
-    <t>1,306 (439-2,898)</t>
-  </si>
-  <si>
-    <t>1,773 (593-3,964)</t>
-  </si>
-  <si>
-    <t>1,719 (625-3,675)</t>
-  </si>
-  <si>
-    <t>2,983 (1,115-6,341)</t>
-  </si>
-  <si>
-    <t>4,027 (1,481-8,294)</t>
-  </si>
-  <si>
-    <t>1,802 (632-3,866)</t>
-  </si>
-  <si>
-    <t>3,141 (1,115-6,813)</t>
-  </si>
-  <si>
-    <t>4,189 (1,493-9,069)</t>
-  </si>
-  <si>
-    <t>200 (87.8-470)</t>
-  </si>
-  <si>
-    <t>380 (152-822)</t>
-  </si>
-  <si>
-    <t>497 (203-1,097)</t>
-  </si>
-  <si>
-    <t>286 (99.3-732)</t>
-  </si>
-  <si>
-    <t>558 (177-1,388)</t>
-  </si>
-  <si>
-    <t>771 (241-2,018)</t>
-  </si>
-  <si>
-    <t>1,264 (424-2,951)</t>
-  </si>
-  <si>
-    <t>2,222 (749-5,155)</t>
-  </si>
-  <si>
-    <t>2,943 (1,015-6,886)</t>
-  </si>
-  <si>
-    <t>1,322 (438-3,189)</t>
-  </si>
-  <si>
-    <t>2,292 (762-5,625)</t>
-  </si>
-  <si>
-    <t>3,041 (1,025-7,531)</t>
-  </si>
-  <si>
-    <t>149 (41.3-285)</t>
-  </si>
-  <si>
-    <t>233 (68.8-498)</t>
-  </si>
-  <si>
-    <t>319 (88.3-664)</t>
-  </si>
-  <si>
-    <t>368 (154-873)</t>
-  </si>
-  <si>
-    <t>702 (280-1,692)</t>
-  </si>
-  <si>
-    <t>1,001 (398-2,474)</t>
-  </si>
-  <si>
-    <t>167 (56.5-320)</t>
-  </si>
-  <si>
-    <t>272 (94.5-565)</t>
-  </si>
-  <si>
-    <t>363 (124-746)</t>
-  </si>
-  <si>
-    <t>385 (157-919)</t>
-  </si>
-  <si>
-    <t>722 (292-1,770)</t>
-  </si>
-  <si>
-    <t>1,023 (404-2,551)</t>
-  </si>
-  <si>
-    <t>55 (19.9-119)</t>
-  </si>
-  <si>
-    <t>96 (34.8-211)</t>
-  </si>
-  <si>
-    <t>128 (46.8-284)</t>
-  </si>
-  <si>
-    <t>1,178 (438-3,002)</t>
-  </si>
-  <si>
-    <t>2,323 (864-5,933)</t>
-  </si>
-  <si>
-    <t>3,450 (1,280-8,808)</t>
-  </si>
-  <si>
-    <t>222 (75.0-671)</t>
-  </si>
-  <si>
-    <t>420 (137-1,203)</t>
-  </si>
-  <si>
-    <t>592 (192-1,630)</t>
-  </si>
-  <si>
-    <t>1,310 (490-3,441)</t>
-  </si>
-  <si>
-    <t>2,514 (930-6,532)</t>
-  </si>
-  <si>
-    <t>3,626 (1,332-9,353)</t>
+    <t>738 (284-1,436)</t>
+  </si>
+  <si>
+    <t>1,249 (495-2,475)</t>
+  </si>
+  <si>
+    <t>1,620 (646-3,267)</t>
+  </si>
+  <si>
+    <t>787 (287-1,522)</t>
+  </si>
+  <si>
+    <t>1,338 (505-2,685)</t>
+  </si>
+  <si>
+    <t>1,808 (685-3,606)</t>
+  </si>
+  <si>
+    <t>1,848 (812-3,116)</t>
+  </si>
+  <si>
+    <t>3,073 (1,412-5,386)</t>
+  </si>
+  <si>
+    <t>4,103 (1,903-7,119)</t>
+  </si>
+  <si>
+    <t>1,895 (820-3,203)</t>
+  </si>
+  <si>
+    <t>3,152 (1,427-5,593)</t>
+  </si>
+  <si>
+    <t>4,191 (1,905-7,336)</t>
+  </si>
+  <si>
+    <t>238 (116-470)</t>
+  </si>
+  <si>
+    <t>449 (199-836)</t>
+  </si>
+  <si>
+    <t>601 (265-1,107)</t>
+  </si>
+  <si>
+    <t>296 (127-598)</t>
+  </si>
+  <si>
+    <t>565 (228-1,100)</t>
+  </si>
+  <si>
+    <t>772 (313-1,534)</t>
+  </si>
+  <si>
+    <t>1,341 (564-2,438)</t>
+  </si>
+  <si>
+    <t>2,350 (993-4,196)</t>
+  </si>
+  <si>
+    <t>3,069 (1,341-5,511)</t>
+  </si>
+  <si>
+    <t>1,373 (574-2,543)</t>
+  </si>
+  <si>
+    <t>2,410 (1,012-4,388)</t>
+  </si>
+  <si>
+    <t>3,139 (1,371-5,835)</t>
+  </si>
+  <si>
+    <t>161 (49.2-330)</t>
+  </si>
+  <si>
+    <t>275 (82.0-569)</t>
+  </si>
+  <si>
+    <t>374 (105-744)</t>
+  </si>
+  <si>
+    <t>344 (154-643)</t>
+  </si>
+  <si>
+    <t>632 (283-1,212)</t>
+  </si>
+  <si>
+    <t>899 (395-1,740)</t>
+  </si>
+  <si>
+    <t>174 (59.3-341)</t>
+  </si>
+  <si>
+    <t>292 (101-592)</t>
+  </si>
+  <si>
+    <t>401 (130-793)</t>
+  </si>
+  <si>
+    <t>355 (158-662)</t>
+  </si>
+  <si>
+    <t>646 (287-1,244)</t>
+  </si>
+  <si>
+    <t>909 (399-1,773)</t>
+  </si>
+  <si>
+    <t>35 (17.7-82.3)</t>
+  </si>
+  <si>
+    <t>70 (31.8-145)</t>
+  </si>
+  <si>
+    <t>95 (43.1-195)</t>
+  </si>
+  <si>
+    <t>946 (423-1,929)</t>
+  </si>
+  <si>
+    <t>1,878 (836-3,811)</t>
+  </si>
+  <si>
+    <t>2,791 (1,241-5,659)</t>
+  </si>
+  <si>
+    <t>146 (65.5-350)</t>
+  </si>
+  <si>
+    <t>279 (120-624)</t>
+  </si>
+  <si>
+    <t>392 (165-852)</t>
+  </si>
+  <si>
+    <t>1,034 (459-2,134)</t>
+  </si>
+  <si>
+    <t>2,003 (886-4,089)</t>
+  </si>
+  <si>
+    <t>2,910 (1,288-5,911)</t>
   </si>
 </sst>
 </file>

</xml_diff>